<commit_message>
chore: sync latest local changes to repository
</commit_message>
<xml_diff>
--- a/Recon_Report_tempDocument_1_1765880545323.csv.xlsx
+++ b/Recon_Report_tempDocument_1_1765880545323.csv.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary Dashboard" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reconciliation Details" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Summary Dashboard" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Reconciliation Details" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -40,7 +40,7 @@
       <color rgb="00FFFFFF"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="6">
     <fill>
       <patternFill/>
     </fill>
@@ -59,6 +59,18 @@
         <bgColor rgb="004472C4"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFC7CE"/>
+        <bgColor rgb="00FFC7CE"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFEB9C"/>
+        <bgColor rgb="00FFEB9C"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -72,7 +84,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -80,6 +92,8 @@
     <xf numFmtId="0" fontId="3" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -157,13 +171,13 @@
 </file>
 
 <file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:bodyPr/>
+          <a:p>
             <a:pPr>
               <a:defRPr/>
             </a:pPr>
@@ -186,7 +200,7 @@
             </strRef>
           </tx>
           <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:ln>
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
@@ -214,13 +228,13 @@
 </file>
 
 <file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:bodyPr/>
+          <a:p>
             <a:pPr>
               <a:defRPr/>
             </a:pPr>
@@ -244,7 +258,7 @@
             </strRef>
           </tx>
           <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:ln>
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
@@ -293,7 +307,7 @@
 </file>
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
       <col>3</col>
@@ -308,9 +322,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+      <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+          <c:chart r:id="rId1"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -330,9 +344,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+      <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId2"/>
+          <c:chart r:id="rId2"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -663,7 +677,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-02-06 09:45:59</t>
+          <t>2026-02-13 13:54:41</t>
         </is>
       </c>
       <c r="Z2" t="inlineStr">
@@ -672,7 +686,7 @@
         </is>
       </c>
       <c r="AA2" t="n">
-        <v>109</v>
+        <v>70</v>
       </c>
     </row>
     <row r="3">
@@ -684,7 +698,7 @@
         </is>
       </c>
       <c r="AA3" t="n">
-        <v>0</v>
+        <v>16</v>
       </c>
     </row>
     <row r="4">
@@ -700,7 +714,7 @@
         </is>
       </c>
       <c r="AA4" t="n">
-        <v>0</v>
+        <v>23</v>
       </c>
     </row>
     <row r="5">
@@ -718,7 +732,7 @@
         </is>
       </c>
       <c r="AA5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="6">
@@ -768,7 +782,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>109</v>
+        <v>70</v>
       </c>
       <c r="Z9" t="inlineStr">
         <is>
@@ -786,7 +800,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>0</v>
+        <v>16</v>
       </c>
     </row>
     <row r="11">
@@ -796,7 +810,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>0</v>
+        <v>23</v>
       </c>
     </row>
     <row r="12">
@@ -806,7 +820,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="13">
@@ -821,7 +835,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>100.00%</t>
+          <t>64.22%</t>
         </is>
       </c>
     </row>
@@ -872,15 +886,15 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F2"/>
+  <dimension ref="A1:F46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="22" customWidth="1" min="1" max="1"/>
-    <col width="7" customWidth="1" min="2" max="2"/>
-    <col width="16" customWidth="1" min="3" max="3"/>
-    <col width="16" customWidth="1" min="4" max="4"/>
-    <col width="12" customWidth="1" min="5" max="5"/>
-    <col width="9" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="21" customWidth="1" min="2" max="2"/>
+    <col width="25" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="11" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -916,34 +930,1106 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>No differences found</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>MATCHED</t>
+      <c r="A2" s="5" t="inlineStr">
+        <is>
+          <t>699449</t>
+        </is>
+      </c>
+      <c r="B2" s="5" t="inlineStr">
+        <is>
+          <t>Nominal</t>
+        </is>
+      </c>
+      <c r="C2" s="5" t="n">
+        <v>2000000000</v>
+      </c>
+      <c r="D2" s="5" t="n">
+        <v>37863717</v>
+      </c>
+      <c r="E2" s="5" t="inlineStr">
+        <is>
+          <t>Value Mismatch</t>
+        </is>
+      </c>
+      <c r="F2" s="5" t="inlineStr">
+        <is>
+          <t>MISMATCH</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="5" t="inlineStr">
+        <is>
+          <t>699449</t>
+        </is>
+      </c>
+      <c r="B3" s="5" t="inlineStr">
+        <is>
+          <t>Trade Price</t>
+        </is>
+      </c>
+      <c r="C3" s="5" t="n">
+        <v>105288461.53846</v>
+      </c>
+      <c r="D3" s="5" t="n">
+        <v>105288461.5</v>
+      </c>
+      <c r="E3" s="5" t="inlineStr">
+        <is>
+          <t>Value Mismatch</t>
+        </is>
+      </c>
+      <c r="F3" s="5" t="inlineStr">
+        <is>
+          <t>MISMATCH</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>698853</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="inlineStr">
+        <is>
+          <t>Quantity</t>
+        </is>
+      </c>
+      <c r="C4" s="5" t="n">
+        <v>350000</v>
+      </c>
+      <c r="D4" s="5" t="n">
+        <v>328974</v>
+      </c>
+      <c r="E4" s="5" t="inlineStr">
+        <is>
+          <t>Value Mismatch</t>
+        </is>
+      </c>
+      <c r="F4" s="5" t="inlineStr">
+        <is>
+          <t>MISMATCH</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>699400</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="inlineStr">
+        <is>
+          <t>CounterParty</t>
+        </is>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>CRDB BANK TZ</t>
+        </is>
+      </c>
+      <c r="D5" s="5" t="inlineStr">
+        <is>
+          <t>CRDB</t>
+        </is>
+      </c>
+      <c r="E5" s="5" t="inlineStr">
+        <is>
+          <t>Value Mismatch</t>
+        </is>
+      </c>
+      <c r="F5" s="5" t="inlineStr">
+        <is>
+          <t>MISMATCH</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>699400</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="inlineStr">
+        <is>
+          <t>Entered User</t>
+        </is>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>calypso</t>
+        </is>
+      </c>
+      <c r="D6" s="5" t="inlineStr">
+        <is>
+          <t>admin</t>
+        </is>
+      </c>
+      <c r="E6" s="5" t="inlineStr">
+        <is>
+          <t>Value Mismatch</t>
+        </is>
+      </c>
+      <c r="F6" s="5" t="inlineStr">
+        <is>
+          <t>MISMATCH</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>699118</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="inlineStr">
+        <is>
+          <t>Quantity</t>
+        </is>
+      </c>
+      <c r="C7" s="5" t="n">
+        <v>10000000</v>
+      </c>
+      <c r="D7" s="5" t="n">
+        <v>874878742</v>
+      </c>
+      <c r="E7" s="5" t="inlineStr">
+        <is>
+          <t>Value Mismatch</t>
+        </is>
+      </c>
+      <c r="F7" s="5" t="inlineStr">
+        <is>
+          <t>MISMATCH</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="5" t="inlineStr">
+        <is>
+          <t>698857</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="inlineStr">
+        <is>
+          <t>Entered User</t>
+        </is>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>phayghaimo</t>
+        </is>
+      </c>
+      <c r="D8" s="5" t="inlineStr">
+        <is>
+          <t>play</t>
+        </is>
+      </c>
+      <c r="E8" s="5" t="inlineStr">
+        <is>
+          <t>Value Mismatch</t>
+        </is>
+      </c>
+      <c r="F8" s="5" t="inlineStr">
+        <is>
+          <t>MISMATCH</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>698067</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="inlineStr">
+        <is>
+          <t>Trade Price</t>
+        </is>
+      </c>
+      <c r="C9" s="5" t="n">
+        <v>105288461.53846</v>
+      </c>
+      <c r="D9" s="5" t="n">
+        <v>105288461.5</v>
+      </c>
+      <c r="E9" s="5" t="inlineStr">
+        <is>
+          <t>Value Mismatch</t>
+        </is>
+      </c>
+      <c r="F9" s="5" t="inlineStr">
+        <is>
+          <t>MISMATCH</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="5" t="inlineStr">
+        <is>
+          <t>699120</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="inlineStr">
+        <is>
+          <t>Nominal</t>
+        </is>
+      </c>
+      <c r="C10" s="5" t="n">
+        <v>2000000000</v>
+      </c>
+      <c r="D10" s="5" t="n">
+        <v>23873288</v>
+      </c>
+      <c r="E10" s="5" t="inlineStr">
+        <is>
+          <t>Value Mismatch</t>
+        </is>
+      </c>
+      <c r="F10" s="5" t="inlineStr">
+        <is>
+          <t>MISMATCH</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="5" t="inlineStr">
+        <is>
+          <t>699120</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="inlineStr">
+        <is>
+          <t>Trade Price</t>
+        </is>
+      </c>
+      <c r="C11" s="5" t="n">
+        <v>100274725.27473</v>
+      </c>
+      <c r="D11" s="5" t="n">
+        <v>100274725.3</v>
+      </c>
+      <c r="E11" s="5" t="inlineStr">
+        <is>
+          <t>Value Mismatch</t>
+        </is>
+      </c>
+      <c r="F11" s="5" t="inlineStr">
+        <is>
+          <t>MISMATCH</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="5" t="inlineStr">
+        <is>
+          <t>699414</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="inlineStr">
+        <is>
+          <t>Product Type</t>
+        </is>
+      </c>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>UnitizedFund</t>
+        </is>
+      </c>
+      <c r="D12" s="5" t="inlineStr">
+        <is>
+          <t>CA</t>
+        </is>
+      </c>
+      <c r="E12" s="5" t="inlineStr">
+        <is>
+          <t>Value Mismatch</t>
+        </is>
+      </c>
+      <c r="F12" s="5" t="inlineStr">
+        <is>
+          <t>MISMATCH</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="5" t="inlineStr">
+        <is>
+          <t>698932</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="inlineStr">
+        <is>
+          <t>Nominal</t>
+        </is>
+      </c>
+      <c r="C13" s="5" t="n">
+        <v>305460</v>
+      </c>
+      <c r="D13" s="5" t="n">
+        <v>77585</v>
+      </c>
+      <c r="E13" s="5" t="inlineStr">
+        <is>
+          <t>Value Mismatch</t>
+        </is>
+      </c>
+      <c r="F13" s="5" t="inlineStr">
+        <is>
+          <t>MISMATCH</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="5" t="inlineStr">
+        <is>
+          <t>698910</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="inlineStr">
+        <is>
+          <t>Product Description</t>
+        </is>
+      </c>
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>FX/USD/TZS</t>
+        </is>
+      </c>
+      <c r="D14" s="5" t="inlineStr">
+        <is>
+          <t>FX/FX</t>
+        </is>
+      </c>
+      <c r="E14" s="5" t="inlineStr">
+        <is>
+          <t>Value Mismatch</t>
+        </is>
+      </c>
+      <c r="F14" s="5" t="inlineStr">
+        <is>
+          <t>MISMATCH</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="5" t="inlineStr">
+        <is>
+          <t>698068</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="inlineStr">
+        <is>
+          <t>Trade Price</t>
+        </is>
+      </c>
+      <c r="C15" s="5" t="n">
+        <v>105288461.53846</v>
+      </c>
+      <c r="D15" s="5" t="n">
+        <v>105288461.5</v>
+      </c>
+      <c r="E15" s="5" t="inlineStr">
+        <is>
+          <t>Value Mismatch</t>
+        </is>
+      </c>
+      <c r="F15" s="5" t="inlineStr">
+        <is>
+          <t>MISMATCH</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="5" t="inlineStr">
+        <is>
+          <t>699393</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="inlineStr">
+        <is>
+          <t>Book</t>
+        </is>
+      </c>
+      <c r="C16" s="5" t="inlineStr">
+        <is>
+          <t>BI_FI_AC_Bond</t>
+        </is>
+      </c>
+      <c r="D16" s="5" t="inlineStr">
+        <is>
+          <t>BI_FI</t>
+        </is>
+      </c>
+      <c r="E16" s="5" t="inlineStr">
+        <is>
+          <t>Value Mismatch</t>
+        </is>
+      </c>
+      <c r="F16" s="5" t="inlineStr">
+        <is>
+          <t>MISMATCH</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="5" t="inlineStr">
+        <is>
+          <t>699393</t>
+        </is>
+      </c>
+      <c r="B17" s="5" t="inlineStr">
+        <is>
+          <t>Notional</t>
+        </is>
+      </c>
+      <c r="C17" s="5" t="n">
+        <v>1000000000</v>
+      </c>
+      <c r="D17" s="5" t="n">
+        <v>200000000</v>
+      </c>
+      <c r="E17" s="5" t="inlineStr">
+        <is>
+          <t>Value Mismatch</t>
+        </is>
+      </c>
+      <c r="F17" s="5" t="inlineStr">
+        <is>
+          <t>MISMATCH</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="5" t="inlineStr">
+        <is>
+          <t>699448</t>
+        </is>
+      </c>
+      <c r="B18" s="5" t="inlineStr">
+        <is>
+          <t>Trade Price</t>
+        </is>
+      </c>
+      <c r="C18" s="5" t="n">
+        <v>105288461.53846</v>
+      </c>
+      <c r="D18" s="5" t="n">
+        <v>105288461.5</v>
+      </c>
+      <c r="E18" s="5" t="inlineStr">
+        <is>
+          <t>Value Mismatch</t>
+        </is>
+      </c>
+      <c r="F18" s="5" t="inlineStr">
+        <is>
+          <t>MISMATCH</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="5" t="inlineStr">
+        <is>
+          <t>699442</t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="inlineStr">
+        <is>
+          <t>Trade Currency</t>
+        </is>
+      </c>
+      <c r="C19" s="5" t="inlineStr">
+        <is>
+          <t>BIF</t>
+        </is>
+      </c>
+      <c r="D19" s="5" t="inlineStr">
+        <is>
+          <t>TZS</t>
+        </is>
+      </c>
+      <c r="E19" s="5" t="inlineStr">
+        <is>
+          <t>Value Mismatch</t>
+        </is>
+      </c>
+      <c r="F19" s="5" t="inlineStr">
+        <is>
+          <t>MISMATCH</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="5" t="inlineStr">
+        <is>
+          <t>699428</t>
+        </is>
+      </c>
+      <c r="B20" s="5" t="inlineStr">
+        <is>
+          <t>Product Description</t>
+        </is>
+      </c>
+      <c r="C20" s="5" t="inlineStr">
+        <is>
+          <t>Inuka Money Market Fund</t>
+        </is>
+      </c>
+      <c r="D20" s="5" t="inlineStr">
+        <is>
+          <t>Cash</t>
+        </is>
+      </c>
+      <c r="E20" s="5" t="inlineStr">
+        <is>
+          <t>Value Mismatch</t>
+        </is>
+      </c>
+      <c r="F20" s="5" t="inlineStr">
+        <is>
+          <t>MISMATCH</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="5" t="inlineStr">
+        <is>
+          <t>698892</t>
+        </is>
+      </c>
+      <c r="B21" s="5" t="inlineStr">
+        <is>
+          <t>Nominal</t>
+        </is>
+      </c>
+      <c r="C21" s="5" t="n">
+        <v>3000000000</v>
+      </c>
+      <c r="D21" s="5" t="n">
+        <v>3743234</v>
+      </c>
+      <c r="E21" s="5" t="inlineStr">
+        <is>
+          <t>Value Mismatch</t>
+        </is>
+      </c>
+      <c r="F21" s="5" t="inlineStr">
+        <is>
+          <t>MISMATCH</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="5" t="inlineStr">
+        <is>
+          <t>698892</t>
+        </is>
+      </c>
+      <c r="B22" s="5" t="inlineStr">
+        <is>
+          <t>CounterParty</t>
+        </is>
+      </c>
+      <c r="C22" s="5" t="inlineStr">
+        <is>
+          <t>CRDB BANK TZ</t>
+        </is>
+      </c>
+      <c r="D22" s="5" t="inlineStr">
+        <is>
+          <t>CRDB+B62 BANK TZ</t>
+        </is>
+      </c>
+      <c r="E22" s="5" t="inlineStr">
+        <is>
+          <t>Value Mismatch</t>
+        </is>
+      </c>
+      <c r="F22" s="5" t="inlineStr">
+        <is>
+          <t>MISMATCH</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="6" t="inlineStr">
+        <is>
+          <t>698087</t>
+        </is>
+      </c>
+      <c r="B23" s="6" t="inlineStr"/>
+      <c r="C23" s="6" t="inlineStr"/>
+      <c r="D23" s="6" t="inlineStr"/>
+      <c r="E23" s="6" t="inlineStr">
+        <is>
+          <t>Missing in B</t>
+        </is>
+      </c>
+      <c r="F23" s="6" t="inlineStr">
+        <is>
+          <t>ONLY IN A</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="6" t="inlineStr">
+        <is>
+          <t>698210</t>
+        </is>
+      </c>
+      <c r="B24" s="6" t="inlineStr"/>
+      <c r="C24" s="6" t="inlineStr"/>
+      <c r="D24" s="6" t="inlineStr"/>
+      <c r="E24" s="6" t="inlineStr">
+        <is>
+          <t>Missing in B</t>
+        </is>
+      </c>
+      <c r="F24" s="6" t="inlineStr">
+        <is>
+          <t>ONLY IN A</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="6" t="inlineStr">
+        <is>
+          <t>698801</t>
+        </is>
+      </c>
+      <c r="B25" s="6" t="inlineStr"/>
+      <c r="C25" s="6" t="inlineStr"/>
+      <c r="D25" s="6" t="inlineStr"/>
+      <c r="E25" s="6" t="inlineStr">
+        <is>
+          <t>Missing in B</t>
+        </is>
+      </c>
+      <c r="F25" s="6" t="inlineStr">
+        <is>
+          <t>ONLY IN A</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="6" t="inlineStr">
+        <is>
+          <t>698396</t>
+        </is>
+      </c>
+      <c r="B26" s="6" t="inlineStr"/>
+      <c r="C26" s="6" t="inlineStr"/>
+      <c r="D26" s="6" t="inlineStr"/>
+      <c r="E26" s="6" t="inlineStr">
+        <is>
+          <t>Missing in B</t>
+        </is>
+      </c>
+      <c r="F26" s="6" t="inlineStr">
+        <is>
+          <t>ONLY IN A</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="6" t="inlineStr">
+        <is>
+          <t>698317</t>
+        </is>
+      </c>
+      <c r="B27" s="6" t="inlineStr"/>
+      <c r="C27" s="6" t="inlineStr"/>
+      <c r="D27" s="6" t="inlineStr"/>
+      <c r="E27" s="6" t="inlineStr">
+        <is>
+          <t>Missing in B</t>
+        </is>
+      </c>
+      <c r="F27" s="6" t="inlineStr">
+        <is>
+          <t>ONLY IN A</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="6" t="inlineStr">
+        <is>
+          <t>698848</t>
+        </is>
+      </c>
+      <c r="B28" s="6" t="inlineStr"/>
+      <c r="C28" s="6" t="inlineStr"/>
+      <c r="D28" s="6" t="inlineStr"/>
+      <c r="E28" s="6" t="inlineStr">
+        <is>
+          <t>Missing in B</t>
+        </is>
+      </c>
+      <c r="F28" s="6" t="inlineStr">
+        <is>
+          <t>ONLY IN A</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="6" t="inlineStr">
+        <is>
+          <t>698198</t>
+        </is>
+      </c>
+      <c r="B29" s="6" t="inlineStr"/>
+      <c r="C29" s="6" t="inlineStr"/>
+      <c r="D29" s="6" t="inlineStr"/>
+      <c r="E29" s="6" t="inlineStr">
+        <is>
+          <t>Missing in B</t>
+        </is>
+      </c>
+      <c r="F29" s="6" t="inlineStr">
+        <is>
+          <t>ONLY IN A</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="6" t="inlineStr">
+        <is>
+          <t>698083</t>
+        </is>
+      </c>
+      <c r="B30" s="6" t="inlineStr"/>
+      <c r="C30" s="6" t="inlineStr"/>
+      <c r="D30" s="6" t="inlineStr"/>
+      <c r="E30" s="6" t="inlineStr">
+        <is>
+          <t>Missing in B</t>
+        </is>
+      </c>
+      <c r="F30" s="6" t="inlineStr">
+        <is>
+          <t>ONLY IN A</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="6" t="inlineStr">
+        <is>
+          <t>698102</t>
+        </is>
+      </c>
+      <c r="B31" s="6" t="inlineStr"/>
+      <c r="C31" s="6" t="inlineStr"/>
+      <c r="D31" s="6" t="inlineStr"/>
+      <c r="E31" s="6" t="inlineStr">
+        <is>
+          <t>Missing in B</t>
+        </is>
+      </c>
+      <c r="F31" s="6" t="inlineStr">
+        <is>
+          <t>ONLY IN A</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="6" t="inlineStr">
+        <is>
+          <t>698092</t>
+        </is>
+      </c>
+      <c r="B32" s="6" t="inlineStr"/>
+      <c r="C32" s="6" t="inlineStr"/>
+      <c r="D32" s="6" t="inlineStr"/>
+      <c r="E32" s="6" t="inlineStr">
+        <is>
+          <t>Missing in B</t>
+        </is>
+      </c>
+      <c r="F32" s="6" t="inlineStr">
+        <is>
+          <t>ONLY IN A</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="6" t="inlineStr">
+        <is>
+          <t>698212</t>
+        </is>
+      </c>
+      <c r="B33" s="6" t="inlineStr"/>
+      <c r="C33" s="6" t="inlineStr"/>
+      <c r="D33" s="6" t="inlineStr"/>
+      <c r="E33" s="6" t="inlineStr">
+        <is>
+          <t>Missing in B</t>
+        </is>
+      </c>
+      <c r="F33" s="6" t="inlineStr">
+        <is>
+          <t>ONLY IN A</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="6" t="inlineStr">
+        <is>
+          <t>698070</t>
+        </is>
+      </c>
+      <c r="B34" s="6" t="inlineStr"/>
+      <c r="C34" s="6" t="inlineStr"/>
+      <c r="D34" s="6" t="inlineStr"/>
+      <c r="E34" s="6" t="inlineStr">
+        <is>
+          <t>Missing in B</t>
+        </is>
+      </c>
+      <c r="F34" s="6" t="inlineStr">
+        <is>
+          <t>ONLY IN A</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="6" t="inlineStr">
+        <is>
+          <t>698830</t>
+        </is>
+      </c>
+      <c r="B35" s="6" t="inlineStr"/>
+      <c r="C35" s="6" t="inlineStr"/>
+      <c r="D35" s="6" t="inlineStr"/>
+      <c r="E35" s="6" t="inlineStr">
+        <is>
+          <t>Missing in B</t>
+        </is>
+      </c>
+      <c r="F35" s="6" t="inlineStr">
+        <is>
+          <t>ONLY IN A</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="6" t="inlineStr">
+        <is>
+          <t>698103</t>
+        </is>
+      </c>
+      <c r="B36" s="6" t="inlineStr"/>
+      <c r="C36" s="6" t="inlineStr"/>
+      <c r="D36" s="6" t="inlineStr"/>
+      <c r="E36" s="6" t="inlineStr">
+        <is>
+          <t>Missing in B</t>
+        </is>
+      </c>
+      <c r="F36" s="6" t="inlineStr">
+        <is>
+          <t>ONLY IN A</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="6" t="inlineStr">
+        <is>
+          <t>698080</t>
+        </is>
+      </c>
+      <c r="B37" s="6" t="inlineStr"/>
+      <c r="C37" s="6" t="inlineStr"/>
+      <c r="D37" s="6" t="inlineStr"/>
+      <c r="E37" s="6" t="inlineStr">
+        <is>
+          <t>Missing in B</t>
+        </is>
+      </c>
+      <c r="F37" s="6" t="inlineStr">
+        <is>
+          <t>ONLY IN A</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="6" t="inlineStr">
+        <is>
+          <t>698318</t>
+        </is>
+      </c>
+      <c r="B38" s="6" t="inlineStr"/>
+      <c r="C38" s="6" t="inlineStr"/>
+      <c r="D38" s="6" t="inlineStr"/>
+      <c r="E38" s="6" t="inlineStr">
+        <is>
+          <t>Missing in B</t>
+        </is>
+      </c>
+      <c r="F38" s="6" t="inlineStr">
+        <is>
+          <t>ONLY IN A</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="6" t="inlineStr">
+        <is>
+          <t>698796</t>
+        </is>
+      </c>
+      <c r="B39" s="6" t="inlineStr"/>
+      <c r="C39" s="6" t="inlineStr"/>
+      <c r="D39" s="6" t="inlineStr"/>
+      <c r="E39" s="6" t="inlineStr">
+        <is>
+          <t>Missing in B</t>
+        </is>
+      </c>
+      <c r="F39" s="6" t="inlineStr">
+        <is>
+          <t>ONLY IN A</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="6" t="inlineStr">
+        <is>
+          <t>698215</t>
+        </is>
+      </c>
+      <c r="B40" s="6" t="inlineStr"/>
+      <c r="C40" s="6" t="inlineStr"/>
+      <c r="D40" s="6" t="inlineStr"/>
+      <c r="E40" s="6" t="inlineStr">
+        <is>
+          <t>Missing in B</t>
+        </is>
+      </c>
+      <c r="F40" s="6" t="inlineStr">
+        <is>
+          <t>ONLY IN A</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="6" t="inlineStr">
+        <is>
+          <t>698076</t>
+        </is>
+      </c>
+      <c r="B41" s="6" t="inlineStr"/>
+      <c r="C41" s="6" t="inlineStr"/>
+      <c r="D41" s="6" t="inlineStr"/>
+      <c r="E41" s="6" t="inlineStr">
+        <is>
+          <t>Missing in B</t>
+        </is>
+      </c>
+      <c r="F41" s="6" t="inlineStr">
+        <is>
+          <t>ONLY IN A</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="6" t="inlineStr">
+        <is>
+          <t>698402</t>
+        </is>
+      </c>
+      <c r="B42" s="6" t="inlineStr"/>
+      <c r="C42" s="6" t="inlineStr"/>
+      <c r="D42" s="6" t="inlineStr"/>
+      <c r="E42" s="6" t="inlineStr">
+        <is>
+          <t>Missing in B</t>
+        </is>
+      </c>
+      <c r="F42" s="6" t="inlineStr">
+        <is>
+          <t>ONLY IN A</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="6" t="inlineStr">
+        <is>
+          <t>698209</t>
+        </is>
+      </c>
+      <c r="B43" s="6" t="inlineStr"/>
+      <c r="C43" s="6" t="inlineStr"/>
+      <c r="D43" s="6" t="inlineStr"/>
+      <c r="E43" s="6" t="inlineStr">
+        <is>
+          <t>Missing in B</t>
+        </is>
+      </c>
+      <c r="F43" s="6" t="inlineStr">
+        <is>
+          <t>ONLY IN A</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="6" t="inlineStr">
+        <is>
+          <t>698596</t>
+        </is>
+      </c>
+      <c r="B44" s="6" t="inlineStr"/>
+      <c r="C44" s="6" t="inlineStr"/>
+      <c r="D44" s="6" t="inlineStr"/>
+      <c r="E44" s="6" t="inlineStr">
+        <is>
+          <t>Missing in B</t>
+        </is>
+      </c>
+      <c r="F44" s="6" t="inlineStr">
+        <is>
+          <t>ONLY IN A</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="6" t="inlineStr">
+        <is>
+          <t>698211</t>
+        </is>
+      </c>
+      <c r="B45" s="6" t="inlineStr"/>
+      <c r="C45" s="6" t="inlineStr"/>
+      <c r="D45" s="6" t="inlineStr"/>
+      <c r="E45" s="6" t="inlineStr">
+        <is>
+          <t>Missing in B</t>
+        </is>
+      </c>
+      <c r="F45" s="6" t="inlineStr">
+        <is>
+          <t>ONLY IN A</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="6" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="B46" s="6" t="inlineStr"/>
+      <c r="C46" s="6" t="inlineStr"/>
+      <c r="D46" s="6" t="inlineStr"/>
+      <c r="E46" s="6" t="inlineStr">
+        <is>
+          <t>Missing in A</t>
+        </is>
+      </c>
+      <c r="F46" s="6" t="inlineStr">
+        <is>
+          <t>ONLY IN B</t>
         </is>
       </c>
     </row>

</xml_diff>